<commit_message>
Actualizar formato de importación de terceros según especificación del usuario
Cambios implementados:
- Columna "Nombre Código Padre" ahora se mapea directamente a cod_padre
- Columna "V" reconocida como ID opcional (no se usa pero no genera error)
- Columna "nombre" es opcional: si no existe, usa cod_padre como nombre
- Prioridad de mapeo actualizada para "Nombre Código Padre"

Formato de Excel actualizado:
- V: Identificador numérico (columna opcional)
- Nombre Código Padre: Código del tercero (requerida)
- NIT: Número de identificación tributaria (requerida)
- Se Registra: Estado activo/inactivo (opcional, default True)

Archivos modificados:
- tercero_excel_processor.py: Mapeo de columnas actualizado
- generar_excel_terceros_ejemplo.py: Nuevo formato con 4 columnas
- terceros_ejemplo.xlsx: Regenerado con nuevo formato

Nota: Si el Excel no tiene columna "nombre", el sistema usa
automáticamente el valor de "Nombre Código Padre" como nombre del tercero.
</commit_message>
<xml_diff>
--- a/terceros_ejemplo.xlsx
+++ b/terceros_ejemplo.xlsx
@@ -431,36 +431,34 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>cod_padre</t>
+          <t>V</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>nombre</t>
+          <t>Nombre Código Padre</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>nit</t>
+          <t>NIT</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>activo</t>
+          <t>Se Registra</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
         <is>
           <t>T001</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Supermercado La Canasta</t>
-        </is>
-      </c>
       <c r="C2" t="inlineStr">
         <is>
           <t>900123456-1</t>
@@ -471,16 +469,14 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
         <is>
           <t>T002</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Tienda El Ahorro</t>
-        </is>
-      </c>
       <c r="C3" t="inlineStr">
         <is>
           <t>800234567-2</t>
@@ -491,16 +487,14 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
         <is>
           <t>T003</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Distribuidora Los Andes</t>
-        </is>
-      </c>
       <c r="C4" t="inlineStr">
         <is>
           <t>700345678-3</t>
@@ -511,16 +505,14 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
         <is>
           <t>T004</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Café Gourmet del Centro</t>
-        </is>
-      </c>
       <c r="C5" t="inlineStr">
         <is>
           <t>600456789-4</t>
@@ -531,16 +523,14 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
         <is>
           <t>T005</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Supermercado El Éxito</t>
-        </is>
-      </c>
       <c r="C6" t="inlineStr">
         <is>
           <t>890123456-5</t>
@@ -551,16 +541,14 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
         <is>
           <t>T006</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Carrefour Colombia</t>
-        </is>
-      </c>
       <c r="C7" t="inlineStr">
         <is>
           <t>890234567-6</t>
@@ -571,16 +559,14 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
         <is>
           <t>T007</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Tiendas Ara</t>
-        </is>
-      </c>
       <c r="C8" t="inlineStr">
         <is>
           <t>890345678-7</t>
@@ -591,16 +577,14 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
         <is>
           <t>T008</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Olímpica S.A.</t>
-        </is>
-      </c>
       <c r="C9" t="inlineStr">
         <is>
           <t>890456789-8</t>
@@ -611,16 +595,14 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
         <is>
           <t>T009</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>D1 Tiendas</t>
-        </is>
-      </c>
       <c r="C10" t="inlineStr">
         <is>
           <t>890567890-9</t>
@@ -631,16 +613,14 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
         <is>
           <t>T010</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Justo &amp; Bueno</t>
-        </is>
-      </c>
       <c r="C11" t="inlineStr">
         <is>
           <t>890678901-0</t>
@@ -651,14 +631,12 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
         <is>
           <t>T011</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Distribuidora del Valle (Inactivo)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -671,16 +649,14 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
         <is>
           <t>T012</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Makro S.A.</t>
-        </is>
-      </c>
       <c r="C13" t="inlineStr">
         <is>
           <t>890890123-2</t>
@@ -691,16 +667,14 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
         <is>
           <t>T013</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>PriceSmart Colombia</t>
-        </is>
-      </c>
       <c r="C14" t="inlineStr">
         <is>
           <t>890901234-3</t>
@@ -711,16 +685,14 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
         <is>
           <t>T014</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Tiendas Jumbo</t>
-        </is>
-      </c>
       <c r="C15" t="inlineStr">
         <is>
           <t>890012345-4</t>
@@ -731,14 +703,12 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
         <is>
           <t>T015</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Metro Cali</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">

</xml_diff>